<commit_message>
Add Best Builds sheet: 15 winners (best of 3 per arm/prompt) for focused functionality testing
</commit_message>
<xml_diff>
--- a/MVP-Eval-3arm.xlsx
+++ b/MVP-Eval-3arm.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Jobs" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Quality" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Builds" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Jobs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Quality" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,13 +57,13 @@
       <sz val="12"/>
     </font>
     <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="002F5496"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="6">
@@ -142,14 +143,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2985,6 +2986,690 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Best Build per Arm × Prompt — the 15 to functionality-test (best of each 3 by code quality, then spec coverage, then build size)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Best Slug</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Job ID</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Code Q</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>ECU</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Preview URL</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Pass/Fail</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>P1 Task Mgmt</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>kanban-sync</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>98e5fd48-b954-47b2-8a64-706094b79e4e</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>23.16</v>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H4" s="15" t="inlineStr">
+        <is>
+          <t>https://kanban-sync.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>P1 Task Mgmt</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>teamtask-1</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>75c54a5b-5bea-4208-bd55-be080c7f4ba1</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>https://teamtask-1.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>P1 Task Mgmt</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>workflow-pro-6</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>801fb8bb-f01b-40f6-8376-2f19200abe79</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>https://workflow-pro-6.internal.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>P2 PopUp Profit</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>booth-planner-1</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>4cab5e8a-39c6-47d5-805b-6756f86090dc</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>https://booth-planner-1.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>P2 PopUp Profit</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>profit-prep</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>7ab9ef6a-3586-4df7-bf9d-b3be3670426a</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>https://profit-prep.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>P2 PopUp Profit</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>profit-estimator-2</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>1f545f48-600d-490e-a300-73f60e3503eb</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>https://profit-estimator-2.internal.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>P3 Micro-Loans</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>rendoc-loans-4</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>a9dcb442-efb9-4695-a72d-59491ae35736</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>50.54</v>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>https://rendoc-loans-4.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>P3 Micro-Loans</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>rendoc-credit-1</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>e6316c6e-9808-4cc2-a9a1-2e2944103c4f</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>23.59</v>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>https://rendoc-credit-1.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>P3 Micro-Loans</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>micro-lend-hub</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>ca2824b6-39ce-49b2-822c-40f7996ce127</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>35.99</v>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>https://micro-lend-hub.internal.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>P4 Laser-Engrave</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>custom-proof</t>
+        </is>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>c6e82396-1ad2-491a-94cc-353ea125af1a</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>17.31</v>
+      </c>
+      <c r="G16" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>https://custom-proof.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I16" s="14" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>P4 Laser-Engrave</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>design-to-print-1</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>c613a210-a877-46d1-b6f6-48bbaa4637cc</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>17.82</v>
+      </c>
+      <c r="G17" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>https://design-to-print-1.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I17" s="14" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>P4 Laser-Engrave</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>design-engrave</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>cca55d13-6802-44f6-8b41-776128186f8d</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>19.04</v>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>https://design-engrave.internal.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>P5 Context Zero</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>dialogist-fight-1</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>2a70d9a3-3967-43dc-9e86-b8fbef821296</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>33.96</v>
+      </c>
+      <c r="G20" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>https://dialogist-fight-1.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I20" s="14" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>P5 Context Zero</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>context-zero-5</t>
+        </is>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>8da1a228-0b82-44ff-9c9d-8a61c10cc051</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>STARTED</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>https://context-zero-5.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>P5 Context Zero</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>escape-cathedral</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>905438cd-ef82-453e-92b8-356cd0769ce7</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>50.54</v>
+      </c>
+      <c r="G22" s="14" t="inlineStr">
+        <is>
+          <t>RESUMED</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>https://escape-cathedral.internal.stage-preview.emergentagent.com</t>
+        </is>
+      </c>
+      <c r="I22" s="14" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId15"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5801,7 +6486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7667,7 +8352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Preview ECU sheet (ECU-at-first-preview vs 10-credit cap) + conversion data points; per-trajectory subagent dispatch timeline
</commit_message>
<xml_diff>
--- a/MVP-Eval-3arm.xlsx
+++ b/MVP-Eval-3arm.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insights" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Builds" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Jobs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Quality" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview ECU" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Builds" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Jobs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Quality" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -71,7 +72,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -96,6 +97,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FCE9D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -165,11 +176,17 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1197,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1784,61 +1801,85 @@
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>• v2_credit_cap is cheapest overall (avg 16.7 ECU/job) but lowest quality (6.55); it wins ECU on 3/5 prompts.</t>
+          <t>• CONVERSION METRIC (preview before 10-credit cap, via 1st screenshot): Normal 8/15 (53%), v2_credit_cap 13/17 (76%), eph3 10/14 (71%). MVP-split arms get free users to a preview far more often.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
         <is>
-          <t>• eph3 (long-prompt-1) has the HIGHEST quality (7.71 avg) and wins best-quality on 3/5 prompts, at mid cost.</t>
+          <t>• P1 (complex): Normal previews at 10-11.4 ECU (FAILS the cap on all 3) while eph3/v2 preview at 5.5-7 ECU - the core conversion win of MVP-split.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
-          <t>• Normal is the most expensive (23.9 avg) with widest variance; quality 7.23.</t>
+          <t>• P3 (Micro-Loans): EVERY arm fails - first preview at 12-22 ECU, over the 10-cap regardless. Free users churn on P3 no matter the prompt.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>• P1 is the decisive split: v2's best build scored 4/10 (thin) vs Normal &amp; eph3 at 7/10 — v2 under-builds complex apps to hit the cap.</t>
+          <t>• v2_credit_cap is cheapest overall (avg 16.7 ECU/job) but lowest quality (6.55); it wins ECU on 3/5 prompts.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
         <is>
-          <t>• Cost-efficiency (ECU per quality point): v2 2.76 (best $), eph3 2.92, Normal 3.46 (worst).</t>
+          <t>• eph3 (long-prompt-1) has the HIGHEST quality (7.71 avg) and wins best-quality on 3/5 prompts, at mid cost.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
         <is>
-          <t>• v2 is most predictable (ECU stdev 1.8) — the credit cap tightens variance; eph3 spikes on P5 (stdev 21.5, one 50-ECU run).</t>
+          <t>• Normal is the most expensive (23.9 avg) with widest variance; quality 7.23.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
         <is>
+          <t>• P1 is the decisive split: v2's best build scored 4/10 (thin) vs Normal &amp; eph3 at 7/10 — v2 under-builds complex apps to hit the cap.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>• Cost-efficiency (ECU per quality point): v2 2.76 (best $), eph3 2.92, Normal 3.46 (worst).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>• v2 is most predictable (ECU stdev 1.8) — the credit cap tightens variance; eph3 spikes on P5 (stdev 21.5, one 50-ECU run).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
           <t>• eph3 = best quality-for-cost balance; v2 = cheapest but risky on complex prompts; Normal = priciest, no clear win.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="11">
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A33:I33"/>
+    <mergeCell ref="A37:I37"/>
     <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A31:I31"/>
     <mergeCell ref="A34:I34"/>
     <mergeCell ref="A35:I35"/>
+    <mergeCell ref="A38:I38"/>
     <mergeCell ref="A30:I30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1846,6 +1887,2102 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Preview before 10-credit cap — ECU at FIRST screenshot (= app previewable). Free users get 10 credits.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Job ID</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>ECU @ 1st preview</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>#Screenshots</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Total ECU</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Within 10cr?</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Sub-agent dispatches (step@ECU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>kanban-sync</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>98e5fd48-b954-47b2-8a64-706094b79e4e</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F4" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>23.16</v>
+      </c>
+      <c r="I4" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.44  38:testing@17.55</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>project-sync</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>ff6d38e3-a7ba-4be7-9bd3-d068b3bc040e</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>28.57</v>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>3:design@0.55  23:testing@12.24  46:testing@19.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>task-flow-57</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>a2df4e68-83bd-4592-a8da-9c68ee369805</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>11.09</v>
+      </c>
+      <c r="F6" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H6" s="14" t="n">
+        <v>19.48</v>
+      </c>
+      <c r="I6" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.5  28:testing@14.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>booth-planner-1</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>4cab5e8a-39c6-47d5-805b-6756f86090dc</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>11.18</v>
+      </c>
+      <c r="I7" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.44  15:testing@4.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>event-profit-hub</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>31a35f59-0b54-4ab0-8460-be07012901e6</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>4.88</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="I8" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J8" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.45  12:testing@5.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>know-before-show-1</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>fd6a87d5-e834-4615-8f12-8c22a74347b8</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>5.53</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="I9" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.47  15:testing@5.66</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>credit-control</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>e16f0c6a-99c9-44f5-adca-1def18073f05</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>13.94</v>
+      </c>
+      <c r="F10" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="H10" s="14" t="n">
+        <v>41.69</v>
+      </c>
+      <c r="I10" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>2:design@1.16  28:testing@17.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>micro-lending-hub</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>44afcf0c-116b-4f92-81aa-c5c636a89b06</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>22.14</v>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="14" t="n">
+        <v>43.69</v>
+      </c>
+      <c r="I11" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.45  39:testing@26.74</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-loans-4</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>a9dcb442-efb9-4695-a72d-59491ae35736</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>18.84</v>
+      </c>
+      <c r="F12" s="14" t="n">
+        <v>28</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>50.54</v>
+      </c>
+      <c r="I12" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.61  31:testing@19.5  59:testing@40.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>custom-proof</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>c6e82396-1ad2-491a-94cc-353ea125af1a</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>9.15</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>17.31</v>
+      </c>
+      <c r="I13" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.44  19:testing@9.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>engrave-studio-3</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>10cfb936-5fbd-4198-a08e-b42de12431f2</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>23</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>20.78</v>
+      </c>
+      <c r="I14" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.45  25:testing@12.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>vector-create</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>20d5657d-93fd-4562-b875-0b93c31a9cfc</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>7.32</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="I15" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J15" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.49  15:testing@7.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>context-zero-3</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>58fec477-6b64-4f82-b1f0-996d71a8749a</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>18.63</v>
+      </c>
+      <c r="I16" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J16" s="20" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>dialogist-fight-1</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>2a70d9a3-3967-43dc-9e86-b8fbef821296</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>33.96</v>
+      </c>
+      <c r="I17" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J17" s="20" t="inlineStr">
+        <is>
+          <t>76:testing@31.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>prompt-cathedral</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>379095ab-9ecc-43c1-9677-95384bc831c7</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="14" t="n">
+        <v>20.13</v>
+      </c>
+      <c r="I18" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
+        <is>
+          <t>32:testing@14.42</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>project-hub-25</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>2af8df68-1bb9-45bb-ad38-5b7456f0184e</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>6.92</v>
+      </c>
+      <c r="F19" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H19" s="14" t="n">
+        <v>16.35</v>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J19" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.5  16:testing@7.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>teamtask-1</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>75c54a5b-5bea-4208-bd55-be080c7f4ba1</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="G20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>16.88</v>
+      </c>
+      <c r="I20" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J20" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.42  18:testing@6.88</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>workflow-central-2</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>f1959bd6-230e-4e47-86b3-305691d8be15</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>15.97</v>
+      </c>
+      <c r="I21" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J21" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.47  16:testing@5.88  34:testing@12.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>know-before-show-2</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>3645cff0-1c3c-438b-a46a-a5bd9016a351</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="I22" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J22" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.44  11:testing@4.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>profit-prep</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>7ab9ef6a-3586-4df7-bf9d-b3be3670426a</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="I23" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J23" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.51  16:testing@5.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>vendor-calculator-4</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>51d60426-a963-4471-a2b0-5f4635206075</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>7.57</v>
+      </c>
+      <c r="I24" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J24" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.42  14:testing@4.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>micro-loans-admin</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>0cfaeb9d-39fe-45ae-8f6b-fa8fa1439285</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>23</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>17.21</v>
+      </c>
+      <c r="I25" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J25" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.5  11:testing@9.89</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-credit-1</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>e6316c6e-9808-4cc2-a9a1-2e2944103c4f</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="F26" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G26" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>23.59</v>
+      </c>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J26" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.47  17:testing@10.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-portfolio</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>9dec0190-7d4d-4704-bb6b-dff6fa7a9b5b</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>11.98</v>
+      </c>
+      <c r="F27" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>19.16</v>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J27" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.45  14:testing@9.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>create-ship-direct</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>ea163e4a-c6e4-493e-a996-0979f20bacc9</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="F28" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v>20.74</v>
+      </c>
+      <c r="I28" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J28" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.43  18:testing@7.98  37:testing@14.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>custom-maker</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>7564f170-6e9e-4529-a5ca-7411cf42d3a9</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>6.93</v>
+      </c>
+      <c r="F29" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G29" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v>23.27</v>
+      </c>
+      <c r="I29" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J29" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.45  15:testing@7.8  36:testing@15.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>design-to-print-1</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>c613a210-a877-46d1-b6f6-48bbaa4637cc</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="F30" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G30" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H30" s="14" t="n">
+        <v>17.82</v>
+      </c>
+      <c r="I30" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J30" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.5  15:testing@7.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>engrave-studio-4</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>5746d87e-06c6-42ef-a858-b0fa7ee02ca7</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>13.19</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="G31" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H31" s="14" t="n">
+        <v>22.01</v>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J31" s="20" t="inlineStr">
+        <is>
+          <t>3:design@0.56  34:testing@13.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>engrave-studio-5</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>d44d2c97-0a9f-4a85-b8fe-6e7fff6e2fa8</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>7.18</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>21.21</v>
+      </c>
+      <c r="I32" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J32" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.44  18:testing@7.3  52:testing@17.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>personalize-now</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>2cfa1b95-5155-46c5-bd0a-be1220925b62</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>17.22</v>
+      </c>
+      <c r="I33" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J33" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.43  15:testing@7.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>context-zero-5</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>8da1a228-0b82-44ff-9c9d-8a61c10cc051</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J34" s="20" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>escape-ai</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>5a9df756-f574-4bfc-a4fd-1bb86c1fe997</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>7.33</v>
+      </c>
+      <c r="F35" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H35" s="14" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="I35" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J35" s="20" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>kanban-pro-3</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>335a242c-e1a2-4572-8fd3-35a0912464a9</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>7.05</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>14</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>12.31</v>
+      </c>
+      <c r="I36" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J36" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.53  16:testing@7.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>project-flow-9</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>88280310-baed-42e5-97c2-e6ac606bb636</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H37" s="14" t="n">
+        <v>13.32</v>
+      </c>
+      <c r="I37" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J37" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.51  15:testing@6.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>workflow-pro-6</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>801fb8bb-f01b-40f6-8376-2f19200abe79</t>
+        </is>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>6.65</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>11.74</v>
+      </c>
+      <c r="I38" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J38" s="20" t="inlineStr">
+        <is>
+          <t>3:design@0.54  13:testing@6.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>know-before-show-5</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>6f6da5fd-524f-44b7-84da-e027444c9798</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>11.57</v>
+      </c>
+      <c r="I39" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J39" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.51  17:testing@8.27</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>profit-estimator-1</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>9e4b3259-8b8e-4df7-affb-35286b762093</t>
+        </is>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>4.43</v>
+      </c>
+      <c r="F40" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="I40" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J40" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.33  14:testing@4.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>profit-estimator-2</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>1f545f48-600d-490e-a300-73f60e3503eb</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="F41" s="14" t="n">
+        <v>15</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H41" s="14" t="n">
+        <v>10.14</v>
+      </c>
+      <c r="I41" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J41" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.43  17:testing@5.84</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>micro-lend-hub</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>ca2824b6-39ce-49b2-822c-40f7996ce127</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>19.97</v>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>35.99</v>
+      </c>
+      <c r="I42" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J42" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.63  30:testing@20.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>portfolio-pilot</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>93290493-f1ef-402c-b8ce-48c08b0cbcbb</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="n">
+        <v>14.16</v>
+      </c>
+      <c r="F43" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H43" s="14" t="n">
+        <v>30.58</v>
+      </c>
+      <c r="I43" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J43" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.49  22:testing@17.52</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-loans-8</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>9c46c828-8e81-4c87-afb2-c0c9b7b4562e</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="F44" s="14" t="n">
+        <v>17</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H44" s="14" t="n">
+        <v>28.21</v>
+      </c>
+      <c r="I44" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J44" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.44  21:testing@15.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>design-engrave</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>cca55d13-6802-44f6-8b41-776128186f8d</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="F45" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="G45" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" s="14" t="n">
+        <v>19.04</v>
+      </c>
+      <c r="I45" s="19" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J45" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.48  33:testing@14.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>personalize-pro-1</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>ac556cc6-6b8d-4a1c-9b9f-6233c8d49969</t>
+        </is>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="F46" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" s="14" t="n">
+        <v>14.22</v>
+      </c>
+      <c r="I46" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J46" s="20" t="inlineStr">
+        <is>
+          <t>2:design@0.43  20:testing@10.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>context-zero-6</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>d3cd6921-3e6d-488a-895a-f187a4acd31d</t>
+        </is>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>8.710000000000001</v>
+      </c>
+      <c r="F47" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G47" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H47" s="14" t="n">
+        <v>58.23</v>
+      </c>
+      <c r="I47" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J47" s="20" t="inlineStr">
+        <is>
+          <t>47:testing@22.44  86:testing@45.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>dialogist-fight-3</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>dea95022-8eac-4fbe-a6fc-9a3eb501b58f</t>
+        </is>
+      </c>
+      <c r="E48" s="14" t="n">
+        <v>5.82</v>
+      </c>
+      <c r="F48" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G48" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H48" s="14" t="n">
+        <v>9.210000000000001</v>
+      </c>
+      <c r="I48" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J48" s="20" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>escape-cathedral</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>905438cd-ef82-453e-92b8-356cd0769ce7</t>
+        </is>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>9.550000000000001</v>
+      </c>
+      <c r="F49" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="G49" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="H49" s="14" t="n">
+        <v>50.54</v>
+      </c>
+      <c r="I49" s="21" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="J49" s="20" t="inlineStr">
+        <is>
+          <t>96:testing@37.27</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1941,7 +4078,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>https://kanban-sync.stage-preview.emergentagent.com</t>
         </is>
@@ -1973,7 +4110,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E6" s="19" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>https://project-sync.stage-preview.emergentagent.com</t>
         </is>
@@ -2005,7 +4142,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="22" t="inlineStr">
         <is>
           <t>https://task-flow-57.stage-preview.emergentagent.com</t>
         </is>
@@ -2037,7 +4174,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="22" t="inlineStr">
         <is>
           <t>https://project-hub-25.stage-preview.emergentagent.com</t>
         </is>
@@ -2069,7 +4206,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="22" t="inlineStr">
         <is>
           <t>https://teamtask-1.stage-preview.emergentagent.com</t>
         </is>
@@ -2101,7 +4238,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E10" s="19" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>https://workflow-central-2.stage-preview.emergentagent.com</t>
         </is>
@@ -2133,7 +4270,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="22" t="inlineStr">
         <is>
           <t>https://kanban-pro-3.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2165,7 +4302,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>https://project-flow-9.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2197,7 +4334,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E13" s="22" t="inlineStr">
         <is>
           <t>https://workflow-pro-6.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2278,7 +4415,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E17" s="22" t="inlineStr">
         <is>
           <t>https://booth-planner-1.stage-preview.emergentagent.com</t>
         </is>
@@ -2310,7 +4447,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E18" s="22" t="inlineStr">
         <is>
           <t>https://event-profit-hub.stage-preview.emergentagent.com</t>
         </is>
@@ -2342,7 +4479,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E19" s="22" t="inlineStr">
         <is>
           <t>https://know-before-show-1.stage-preview.emergentagent.com</t>
         </is>
@@ -2374,7 +4511,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E20" s="22" t="inlineStr">
         <is>
           <t>https://know-before-show-2.stage-preview.emergentagent.com</t>
         </is>
@@ -2406,7 +4543,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E21" s="19" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>https://profit-prep.stage-preview.emergentagent.com</t>
         </is>
@@ -2438,7 +4575,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E22" s="19" t="inlineStr">
+      <c r="E22" s="22" t="inlineStr">
         <is>
           <t>https://vendor-calculator-4.stage-preview.emergentagent.com</t>
         </is>
@@ -2470,7 +4607,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E23" s="19" t="inlineStr">
+      <c r="E23" s="22" t="inlineStr">
         <is>
           <t>https://know-before-show-5.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2502,7 +4639,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
         <is>
           <t>https://profit-estimator-1.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2534,7 +4671,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E25" s="19" t="inlineStr">
+      <c r="E25" s="22" t="inlineStr">
         <is>
           <t>https://profit-estimator-2.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2615,7 +4752,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr">
+      <c r="E29" s="22" t="inlineStr">
         <is>
           <t>https://credit-control.stage-preview.emergentagent.com</t>
         </is>
@@ -2647,7 +4784,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E30" s="19" t="inlineStr">
+      <c r="E30" s="22" t="inlineStr">
         <is>
           <t>https://micro-lending-hub.stage-preview.emergentagent.com</t>
         </is>
@@ -2679,7 +4816,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E31" s="19" t="inlineStr">
+      <c r="E31" s="22" t="inlineStr">
         <is>
           <t>https://rendoc-loans-4.stage-preview.emergentagent.com</t>
         </is>
@@ -2711,7 +4848,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E32" s="19" t="inlineStr">
+      <c r="E32" s="22" t="inlineStr">
         <is>
           <t>https://micro-loans-admin.stage-preview.emergentagent.com</t>
         </is>
@@ -2743,7 +4880,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E33" s="19" t="inlineStr">
+      <c r="E33" s="22" t="inlineStr">
         <is>
           <t>https://rendoc-credit-1.stage-preview.emergentagent.com</t>
         </is>
@@ -2775,7 +4912,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E34" s="19" t="inlineStr">
+      <c r="E34" s="22" t="inlineStr">
         <is>
           <t>https://rendoc-portfolio.stage-preview.emergentagent.com</t>
         </is>
@@ -2807,7 +4944,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E35" s="19" t="inlineStr">
+      <c r="E35" s="22" t="inlineStr">
         <is>
           <t>https://micro-lend-hub.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2839,7 +4976,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E36" s="19" t="inlineStr">
+      <c r="E36" s="22" t="inlineStr">
         <is>
           <t>https://portfolio-pilot.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2871,7 +5008,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E37" s="19" t="inlineStr">
+      <c r="E37" s="22" t="inlineStr">
         <is>
           <t>https://rendoc-loans-8.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -2952,7 +5089,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E41" s="19" t="inlineStr">
+      <c r="E41" s="22" t="inlineStr">
         <is>
           <t>https://custom-proof.stage-preview.emergentagent.com</t>
         </is>
@@ -2984,7 +5121,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E42" s="19" t="inlineStr">
+      <c r="E42" s="22" t="inlineStr">
         <is>
           <t>https://engrave-studio-3.stage-preview.emergentagent.com</t>
         </is>
@@ -3016,7 +5153,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E43" s="19" t="inlineStr">
+      <c r="E43" s="22" t="inlineStr">
         <is>
           <t>https://vector-create.stage-preview.emergentagent.com</t>
         </is>
@@ -3048,7 +5185,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E44" s="19" t="inlineStr">
+      <c r="E44" s="22" t="inlineStr">
         <is>
           <t>https://create-ship-direct.stage-preview.emergentagent.com</t>
         </is>
@@ -3080,7 +5217,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E45" s="19" t="inlineStr">
+      <c r="E45" s="22" t="inlineStr">
         <is>
           <t>https://custom-maker.stage-preview.emergentagent.com</t>
         </is>
@@ -3112,7 +5249,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E46" s="19" t="inlineStr">
+      <c r="E46" s="22" t="inlineStr">
         <is>
           <t>https://design-to-print-1.stage-preview.emergentagent.com</t>
         </is>
@@ -3144,7 +5281,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E47" s="19" t="inlineStr">
+      <c r="E47" s="22" t="inlineStr">
         <is>
           <t>https://engrave-studio-4.stage-preview.emergentagent.com</t>
         </is>
@@ -3176,7 +5313,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E48" s="19" t="inlineStr">
+      <c r="E48" s="22" t="inlineStr">
         <is>
           <t>https://engrave-studio-5.stage-preview.emergentagent.com</t>
         </is>
@@ -3208,7 +5345,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E49" s="19" t="inlineStr">
+      <c r="E49" s="22" t="inlineStr">
         <is>
           <t>https://personalize-now.stage-preview.emergentagent.com</t>
         </is>
@@ -3240,7 +5377,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E50" s="19" t="inlineStr">
+      <c r="E50" s="22" t="inlineStr">
         <is>
           <t>https://design-engrave.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3272,7 +5409,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E51" s="19" t="inlineStr">
+      <c r="E51" s="22" t="inlineStr">
         <is>
           <t>https://personalize-pro-1.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3353,7 +5490,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E55" s="19" t="inlineStr">
+      <c r="E55" s="22" t="inlineStr">
         <is>
           <t>https://context-zero-3.stage-preview.emergentagent.com</t>
         </is>
@@ -3385,7 +5522,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E56" s="19" t="inlineStr">
+      <c r="E56" s="22" t="inlineStr">
         <is>
           <t>https://dialogist-fight-1.stage-preview.emergentagent.com</t>
         </is>
@@ -3417,7 +5554,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E57" s="19" t="inlineStr">
+      <c r="E57" s="22" t="inlineStr">
         <is>
           <t>https://prompt-cathedral.stage-preview.emergentagent.com</t>
         </is>
@@ -3449,7 +5586,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="E58" s="19" t="inlineStr">
+      <c r="E58" s="22" t="inlineStr">
         <is>
           <t>https://context-zero-5.stage-preview.emergentagent.com</t>
         </is>
@@ -3481,7 +5618,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="E59" s="19" t="inlineStr">
+      <c r="E59" s="22" t="inlineStr">
         <is>
           <t>https://escape-ai.stage-preview.emergentagent.com</t>
         </is>
@@ -3513,7 +5650,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E60" s="19" t="inlineStr">
+      <c r="E60" s="22" t="inlineStr">
         <is>
           <t>https://context-zero-6.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3545,7 +5682,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="E61" s="19" t="inlineStr">
+      <c r="E61" s="22" t="inlineStr">
         <is>
           <t>https://dialogist-fight-3.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3577,7 +5714,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E62" s="19" t="inlineStr">
+      <c r="E62" s="22" t="inlineStr">
         <is>
           <t>https://escape-cathedral.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3649,7 +5786,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3755,7 +5892,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H4" s="19" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>https://kanban-sync.stage-preview.emergentagent.com</t>
         </is>
@@ -3794,7 +5931,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H5" s="19" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>https://teamtask-1.stage-preview.emergentagent.com</t>
         </is>
@@ -3833,7 +5970,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H6" s="19" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>https://workflow-pro-6.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3872,7 +6009,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>https://booth-planner-1.stage-preview.emergentagent.com</t>
         </is>
@@ -3911,7 +6048,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>https://profit-prep.stage-preview.emergentagent.com</t>
         </is>
@@ -3950,7 +6087,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H10" s="19" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>https://profit-estimator-2.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -3989,7 +6126,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H12" s="19" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>https://rendoc-loans-4.stage-preview.emergentagent.com</t>
         </is>
@@ -4028,7 +6165,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H13" s="19" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>https://rendoc-credit-1.stage-preview.emergentagent.com</t>
         </is>
@@ -4067,7 +6204,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H14" s="19" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>https://micro-lend-hub.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -4106,7 +6243,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H16" s="19" t="inlineStr">
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>https://custom-proof.stage-preview.emergentagent.com</t>
         </is>
@@ -4145,7 +6282,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H17" s="19" t="inlineStr">
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>https://design-to-print-1.stage-preview.emergentagent.com</t>
         </is>
@@ -4184,7 +6321,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H18" s="19" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>https://design-engrave.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -4223,7 +6360,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H20" s="19" t="inlineStr">
+      <c r="H20" s="22" t="inlineStr">
         <is>
           <t>https://dialogist-fight-1.stage-preview.emergentagent.com</t>
         </is>
@@ -4262,7 +6399,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="H21" s="19" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>https://context-zero-5.stage-preview.emergentagent.com</t>
         </is>
@@ -4301,7 +6438,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H22" s="19" t="inlineStr">
+      <c r="H22" s="22" t="inlineStr">
         <is>
           <t>https://escape-cathedral.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -4333,7 +6470,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7155,7 +9292,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9021,7 +11158,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Deviation Notes sheet (root cause for every large ECU deviation, cross-arm + within-arm)
</commit_message>
<xml_diff>
--- a/MVP-Eval-3arm.xlsx
+++ b/MVP-Eval-3arm.xlsx
@@ -12,11 +12,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preview ECU" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Methodology" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory Issues" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Builds" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Jobs" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Quality" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deviation Notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Plan" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Best Builds" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Jobs" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Quality" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trajectory" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -138,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -192,6 +193,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1222,6 +1226,1872 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="90" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Arm</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Slug</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Spec</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Arch</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Err</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Sec</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Qual</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Verdict / Top issues</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>kanban-sync</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr"/>
+      <c r="E2" s="14" t="inlineStr"/>
+      <c r="F2" s="14" t="inlineStr"/>
+      <c r="G2" s="14" t="inlineStr"/>
+      <c r="H2" s="14" t="inlineStr"/>
+      <c r="I2" s="14" t="inlineStr"/>
+      <c r="J2" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K2" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L2" s="20" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>project-sync</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr"/>
+      <c r="E3" s="14" t="inlineStr"/>
+      <c r="F3" s="14" t="inlineStr"/>
+      <c r="G3" s="14" t="inlineStr"/>
+      <c r="H3" s="14" t="inlineStr"/>
+      <c r="I3" s="14" t="inlineStr"/>
+      <c r="J3" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K3" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L3" s="20" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>task-flow-57</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr"/>
+      <c r="E4" s="14" t="inlineStr"/>
+      <c r="F4" s="14" t="inlineStr"/>
+      <c r="G4" s="14" t="inlineStr"/>
+      <c r="H4" s="14" t="inlineStr"/>
+      <c r="I4" s="14" t="inlineStr"/>
+      <c r="J4" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K4" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>booth-planner-1</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr"/>
+      <c r="E5" s="14" t="inlineStr"/>
+      <c r="F5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr"/>
+      <c r="H5" s="14" t="inlineStr"/>
+      <c r="I5" s="14" t="inlineStr"/>
+      <c r="J5" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L5" s="20" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>event-profit-hub</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr"/>
+      <c r="E6" s="14" t="inlineStr"/>
+      <c r="F6" s="14" t="inlineStr"/>
+      <c r="G6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr"/>
+      <c r="J6" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L6" s="20" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>know-before-show-1</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr"/>
+      <c r="E7" s="14" t="inlineStr"/>
+      <c r="F7" s="14" t="inlineStr"/>
+      <c r="G7" s="14" t="inlineStr"/>
+      <c r="H7" s="14" t="inlineStr"/>
+      <c r="I7" s="14" t="inlineStr"/>
+      <c r="J7" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K7" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L7" s="20" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>credit-control</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr"/>
+      <c r="E8" s="14" t="inlineStr"/>
+      <c r="F8" s="14" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr"/>
+      <c r="H8" s="14" t="inlineStr"/>
+      <c r="I8" s="14" t="inlineStr"/>
+      <c r="J8" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K8" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L8" s="20" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>micro-lending-hub</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr"/>
+      <c r="E9" s="14" t="inlineStr"/>
+      <c r="F9" s="14" t="inlineStr"/>
+      <c r="G9" s="14" t="inlineStr"/>
+      <c r="H9" s="14" t="inlineStr"/>
+      <c r="I9" s="14" t="inlineStr"/>
+      <c r="J9" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K9" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L9" s="20" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-loans-4</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr"/>
+      <c r="E10" s="14" t="inlineStr"/>
+      <c r="F10" s="14" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr"/>
+      <c r="H10" s="14" t="inlineStr"/>
+      <c r="I10" s="14" t="inlineStr"/>
+      <c r="J10" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K10" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L10" s="20" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>custom-proof</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr"/>
+      <c r="E11" s="14" t="inlineStr"/>
+      <c r="F11" s="14" t="inlineStr"/>
+      <c r="G11" s="14" t="inlineStr"/>
+      <c r="H11" s="14" t="inlineStr"/>
+      <c r="I11" s="14" t="inlineStr"/>
+      <c r="J11" s="14" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="K11" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L11" s="20" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>engrave-studio-3</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr"/>
+      <c r="E12" s="14" t="inlineStr"/>
+      <c r="F12" s="14" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr"/>
+      <c r="H12" s="14" t="inlineStr"/>
+      <c r="I12" s="14" t="inlineStr"/>
+      <c r="J12" s="14" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="K12" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L12" s="20" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>vector-create</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr"/>
+      <c r="E13" s="14" t="inlineStr"/>
+      <c r="F13" s="14" t="inlineStr"/>
+      <c r="G13" s="14" t="inlineStr"/>
+      <c r="H13" s="14" t="inlineStr"/>
+      <c r="I13" s="14" t="inlineStr"/>
+      <c r="J13" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K13" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L13" s="20" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>context-zero-3</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K14" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L14" s="20" t="inlineStr">
+        <is>
+          <t>A polished, feature-complete 3D roguelike vertical slice that covers nearly every spec system with clean engine/UI separation, let down only by a total absence of tests and a vanilla-Three.js (not R3F) implementation. | Issues: Zero tests (empty __init__.py only). Uses globals window.__msgTimer/__dlgTimer (engine.js bridged in Game.jsx:26-32). 1831-line monolith engine. No React error boundary; SSR-off via dynamic import only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>dialogist-fight-1</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K15" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L15" s="20" t="inlineStr">
+        <is>
+          <t>A near-complete, well-structured 3D roguelike that covers nearly every spec system with clean code, held back only by zero automated tests and a few minor dead-code/misleading-UI bugs. | Issues: No tests at all (empty tests dir, template test_result.md). Backend CORS '*' + allow_credentials (unused boilerplate). Dead code: unused dist2, empty gate-poll interval, magic-string 'gate' in castPrompt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Normal (eph1/gflash)</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>prompt-cathedral</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K16" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L16" s="20" t="inlineStr">
+        <is>
+          <t>A feature-complete, well-architected R3F roguelike covering nearly every spec system (movement, dodge, 4 weapons, all prompts, 3 enemies, 4-phase boss, shrines, Model Key gate, full menus), held back only by zero tests and a Next.js-vs-CRA stack deviation. | Issues: No tests at all (empty tests/). Backend CORS allow_credentials=True with '*' origin and os.environ['MONGO_URL'] KeyError risk (dead code). HUD subscribes to full store + per-frame rAF force re-render; updatePickups no-op.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>project-hub-25</t>
+        </is>
+      </c>
+      <c r="D17" s="14" t="inlineStr"/>
+      <c r="E17" s="14" t="inlineStr"/>
+      <c r="F17" s="14" t="inlineStr"/>
+      <c r="G17" s="14" t="inlineStr"/>
+      <c r="H17" s="14" t="inlineStr"/>
+      <c r="I17" s="14" t="inlineStr"/>
+      <c r="J17" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="L17" s="20" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>teamtask-1</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr"/>
+      <c r="E18" s="14" t="inlineStr"/>
+      <c r="F18" s="14" t="inlineStr"/>
+      <c r="G18" s="14" t="inlineStr"/>
+      <c r="H18" s="14" t="inlineStr"/>
+      <c r="I18" s="14" t="inlineStr"/>
+      <c r="J18" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K18" s="14" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="L18" s="20" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>workflow-central-2</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr"/>
+      <c r="E19" s="14" t="inlineStr"/>
+      <c r="F19" s="14" t="inlineStr"/>
+      <c r="G19" s="14" t="inlineStr"/>
+      <c r="H19" s="14" t="inlineStr"/>
+      <c r="I19" s="14" t="inlineStr"/>
+      <c r="J19" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" s="14" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="L19" s="20" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B20" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>know-before-show-2</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr"/>
+      <c r="E20" s="14" t="inlineStr"/>
+      <c r="F20" s="14" t="inlineStr"/>
+      <c r="G20" s="14" t="inlineStr"/>
+      <c r="H20" s="14" t="inlineStr"/>
+      <c r="I20" s="14" t="inlineStr"/>
+      <c r="J20" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K20" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L20" s="20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>profit-prep</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr"/>
+      <c r="E21" s="14" t="inlineStr"/>
+      <c r="F21" s="14" t="inlineStr"/>
+      <c r="G21" s="14" t="inlineStr"/>
+      <c r="H21" s="14" t="inlineStr"/>
+      <c r="I21" s="14" t="inlineStr"/>
+      <c r="J21" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L21" s="20" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>vendor-calculator-4</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr"/>
+      <c r="E22" s="14" t="inlineStr"/>
+      <c r="F22" s="14" t="inlineStr"/>
+      <c r="G22" s="14" t="inlineStr"/>
+      <c r="H22" s="14" t="inlineStr"/>
+      <c r="I22" s="14" t="inlineStr"/>
+      <c r="J22" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K22" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L22" s="20" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>micro-loans-admin</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr"/>
+      <c r="E23" s="14" t="inlineStr"/>
+      <c r="F23" s="14" t="inlineStr"/>
+      <c r="G23" s="14" t="inlineStr"/>
+      <c r="H23" s="14" t="inlineStr"/>
+      <c r="I23" s="14" t="inlineStr"/>
+      <c r="J23" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L23" s="20" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B24" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-credit-1</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr"/>
+      <c r="E24" s="14" t="inlineStr"/>
+      <c r="F24" s="14" t="inlineStr"/>
+      <c r="G24" s="14" t="inlineStr"/>
+      <c r="H24" s="14" t="inlineStr"/>
+      <c r="I24" s="14" t="inlineStr"/>
+      <c r="J24" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K24" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L24" s="20" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-portfolio</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="inlineStr"/>
+      <c r="E25" s="14" t="inlineStr"/>
+      <c r="F25" s="14" t="inlineStr"/>
+      <c r="G25" s="14" t="inlineStr"/>
+      <c r="H25" s="14" t="inlineStr"/>
+      <c r="I25" s="14" t="inlineStr"/>
+      <c r="J25" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L25" s="20" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B26" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>create-ship-direct</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="inlineStr"/>
+      <c r="E26" s="14" t="inlineStr"/>
+      <c r="F26" s="14" t="inlineStr"/>
+      <c r="G26" s="14" t="inlineStr"/>
+      <c r="H26" s="14" t="inlineStr"/>
+      <c r="I26" s="14" t="inlineStr"/>
+      <c r="J26" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K26" s="14" t="inlineStr">
+        <is>
+          <t>Solid</t>
+        </is>
+      </c>
+      <c r="L26" s="20" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>custom-maker</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="inlineStr"/>
+      <c r="E27" s="14" t="inlineStr"/>
+      <c r="F27" s="14" t="inlineStr"/>
+      <c r="G27" s="14" t="inlineStr"/>
+      <c r="H27" s="14" t="inlineStr"/>
+      <c r="I27" s="14" t="inlineStr"/>
+      <c r="J27" s="14" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="K27" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L27" s="20" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B28" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>design-to-print-1</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="inlineStr"/>
+      <c r="E28" s="14" t="inlineStr"/>
+      <c r="F28" s="14" t="inlineStr"/>
+      <c r="G28" s="14" t="inlineStr"/>
+      <c r="H28" s="14" t="inlineStr"/>
+      <c r="I28" s="14" t="inlineStr"/>
+      <c r="J28" s="14" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="K28" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L28" s="20" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>engrave-studio-4</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr"/>
+      <c r="E29" s="14" t="inlineStr"/>
+      <c r="F29" s="14" t="inlineStr"/>
+      <c r="G29" s="14" t="inlineStr"/>
+      <c r="H29" s="14" t="inlineStr"/>
+      <c r="I29" s="14" t="inlineStr"/>
+      <c r="J29" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K29" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L29" s="20" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B30" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>engrave-studio-5</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr"/>
+      <c r="E30" s="14" t="inlineStr"/>
+      <c r="F30" s="14" t="inlineStr"/>
+      <c r="G30" s="14" t="inlineStr"/>
+      <c r="H30" s="14" t="inlineStr"/>
+      <c r="I30" s="14" t="inlineStr"/>
+      <c r="J30" s="14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="K30" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L30" s="20" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>personalize-now</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr"/>
+      <c r="E31" s="14" t="inlineStr"/>
+      <c r="F31" s="14" t="inlineStr"/>
+      <c r="G31" s="14" t="inlineStr"/>
+      <c r="H31" s="14" t="inlineStr"/>
+      <c r="I31" s="14" t="inlineStr"/>
+      <c r="J31" s="14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="K31" s="14" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="L31" s="20" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>context-zero-5</t>
+        </is>
+      </c>
+      <c r="D32" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F32" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G32" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I32" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K32" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L32" s="20" t="inlineStr">
+        <is>
+          <t>A near-complete, well-structured vertical slice that implements virtually the entire spec (movement, dodge, 4 weapons, 4 prompts, 3 enemy types, multi-phase Dialogist boss, pickups, dual upgrade shrine, Model Key gate, connected chambers, full HUD and menus) in clean R3F code, held back mainly by zero automated tests. | Issues: .env committed and not gitignored (localhost Mongo only). CORS defaults to '*' with Allow-Credentials true. State bridged via window.__contextZero global. Dead pickup branches (memory/data never spawned).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>v2_credit_cap (eph2)</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>escape-ai</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H33" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I33" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K33" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L33" s="20" t="inlineStr">
+        <is>
+          <t>A feature-complete, well-structured R3F roguelike covering every spec system (movement, dodge, 4 weapons, 4 prompts, 3 enemies, 4-phase Dialogist, pickups, Data/Humanity shrines, chambers, Model Key gate, full menus) but ships with zero automated tests. | Issues: No tests at all (empty tests/, template test_result.md). Dead code: store.js:319-322 STUN loop does nothing, empty mouse branch. window.__cz_castStun global coupling; boss hardcoded at origin; ~50 unused shadcn components.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>kanban-pro-3</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F34" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I34" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J34" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K34" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L34" s="20" t="inlineStr">
+        <is>
+          <t>A polished, clean implementation of the core CRUD/kanban/dashboard slice with excellent drag-drop and tested isolation, but roughly half the spec breadth (subtasks, comments, search, calendar, dark mode, notifications) is missing. | Issues: CORS allow_origins='*' with allow_credentials=True (insecure/invalid combo); no frontend tests; ~6 spec features absent in both API and UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>project-flow-9</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F35" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H35" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I35" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="J35" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K35" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L35" s="20" t="inlineStr">
+        <is>
+          <t>A clean, well-architected MVP covering auth, projects, task CRUD with properties, kanban drag-drop and dashboard, but it omits roughly half the spec (subtasks, comments, search/filter, calendar, dark mode, notifications). | Issues: CORS allow_origins='*' with allow_credentials=True (env default). Reorder endpoint loops per-item awaits (N writes) without bulk_write. No rate limiting on auth. middleware added after include_router.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>workflow-pro-6</t>
+        </is>
+      </c>
+      <c r="D36" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F36" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H36" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I36" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="J36" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K36" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L36" s="20" t="inlineStr">
+        <is>
+          <t>A clean, well-architected core (auth, task CRUD with properties, owner-scoped queries, polished dnd-kit kanban, dashboard, real backend tests) that omits roughly half the spec's distinctive features—subtasks, comments, calendar, notifications, dark-mode toggle. | Issues: CORS allow_origins='*' with allow_credentials=True (browsers reject; insecure). No login rate limiting. update_task (server.py:316-322) has duplicated/confusing merge logic. due_date stored as string, compared lexicographically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>know-before-show-5</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F37" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G37" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H37" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I37" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J37" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K37" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L37" s="20" t="inlineStr">
+        <is>
+          <t>A polished, feature-complete localStorage-only vendor profit app with sound calculator math, full planner/checklist/dashboard, and clean architecture, held back only by a total absence of frontend tests. | Issues: No frontend tests despite easily testable pure fns (calculator.js, storage.js). Minor: unused imports in Planner; shadowed `num` in formatCurrency; no try/catch on localStorage write (quota).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>profit-estimator-1</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F38" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G38" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="H38" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I38" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J38" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K38" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L38" s="20" t="inlineStr">
+        <is>
+          <t>A clean, fully spec-compliant mobile-first vendor profit app with correct calculator math, full planner, exact 21-item checklist, aggregating dashboard, robust localStorage, and Verbum footer—held back only by zero tests and minor dead code. | Issues: Dashboard.jsx:213-214 dead hidden input sums ev.profitEstimate, a field Planner never writes. tests/ empty—no unit tests for calc math. Dashboard state only read on mount, may show stale data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>profit-estimator-2</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F39" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G39" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="H39" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I39" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="J39" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K39" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L39" s="20" t="inlineStr">
+        <is>
+          <t>A clean, complete, well-structured mobile-first localStorage vendor profit app that covers every spec feature with readable code, though it ships no automated tests. | Issues: No real tests (tests/__init__.py empty). num() silently coerces bad input to 0 with no negative-value guard beyond HTML min. Dashboard upcoming-event date filter is timezone-sensitive (new Date('YYYY-MM-DD')).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>micro-lend-hub</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F40" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G40" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H40" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I40" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="J40" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K40" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L40" s="20" t="inlineStr">
+        <is>
+          <t>A comprehensive, well-architected micro-loans dashboard covering the full spec with clean modular routes, RBAC, risk scoring, and audit logging, held back mainly by CORS/secret hardening gaps. | Issues: CORS allow_origins=* with allow_credentials=True (server.py:80-86); hardcoded JWT_SECRET fallback (auth.py:13); public /applications/intake unbounded; tests are live-URL integration only, no risk-engine unit tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>portfolio-pilot</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F41" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H41" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I41" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="J41" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K41" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L41" s="20" t="inlineStr">
+        <is>
+          <t>A cohesive, well-structured RENDOC micro-loans dashboard covering nearly the entire spec with real RBAC, risk scoring, amortization, collections, audit log and strong integration tests, marred mainly by a stubbed document upload and thin frontend fetch error handling. | Issues: Document upload is a placeholder despite being in spec; frontend load() fetchers lack try/catch (perpetual "Loading"); unauthenticated /seed?force=true wipes all data; CORS=* with allow_credentials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>rendoc-loans-8</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F42" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I42" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="J42" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K42" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L42" s="20" t="inlineStr">
+        <is>
+          <t>A thorough, well-structured full-stack loans platform covering nearly the entire spec (RBAC, pipeline, risk scoring, lifecycle, collections, audit) with broad passing integration tests, held back only by a few security defaults. | Issues: JWT_SECRET hardcoded dev fallback (auth.py:10); CORS allow_origins=* with allow_credentials=True (server.py:1435); upload stores raw file.filename - path traversal risk (server.py:724); reads not scoped to owning officer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>design-engrave</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F43" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G43" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H43" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I43" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="J43" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K43" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L43" s="20" t="inlineStr">
+        <is>
+          <t>A cohesive, well-architected laser-engraving customizer that covers nearly the full spec with a strong live 2D proof flow, production queue, and passing integration tests; main gap is server-side trust of client-supplied prices. | Issues: Server trusts client unit_price/subtotal/total (models.py:93-101); CORS allow_origins=* with allow_credentials=True (server.py:240); default JWT secret in committed .env; GET /orders/{id} unauthenticated (server.py:169).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>personalize-pro-1</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F44" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="G44" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I44" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="J44" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K44" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L44" s="20" t="inlineStr">
+        <is>
+          <t>A clean, cohesive laser-engraving MVP covering catalog, configurator, live 2D proof, volume pricing, checkout, kanban production queue and owner alerts, marred mainly by client-trusted pricing and wildcard CORS. | Issues: server.py:289 trusts client unit_price (price tampering, tiers not re-validated); CORS '*' + allow_credentials True (L594); JWT_SECRET hardcoded fallback (L35).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>context-zero-6</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F45" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G45" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H45" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I45" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J45" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="K45" s="14" t="inlineStr">
+        <is>
+          <t>Acceptable</t>
+        </is>
+      </c>
+      <c r="L45" s="20" t="inlineStr">
+        <is>
+          <t>A complete, well-architected R3F roguelike covering nearly all spec systems (movement, dodge, 4 weapons, 4 enemy types, 4-phase boss, upgrades, key gate, HUD, menus), let down by a non-functional OPEN prompt and a total absence of tests. | Issues: No tests (empty tests/__init__.py, no frontend specs). Dead/abandoned code in levelGen.js:84-96. Boss collider sway math duplicated (Tick.jsx 701-715 vs 752-758). Backend CORS allow_origins='*' + allow_credentials=True (unused boilerplate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>dialogist-fight-3</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="F46" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G46" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="I46" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J46" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K46" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L46" s="20" t="inlineStr">
+        <is>
+          <t>A feature-complete, well-structured 3D roguelike that delivers nearly every spec system (4-phase boss, prompts, 3 enemy types, key gate, dual-path upgrades, full menus) but ships with zero automated tests. | Issues: Empty tests/ dir, no test framework. Minor dead code: unused lineHitsWall, no-op SWARM?1:1 (gameplay.js:672), unused onPause prop, duplicate root route. CORS defaults to '*'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>eph3 (long-prompt-1)</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>escape-cathedral</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="F47" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="G47" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="H47" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="I47" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="K47" s="14" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="L47" s="20" t="inlineStr">
+        <is>
+          <t>A near-complete, cleanly architected R3F roguelike covering essentially every spec system (movement, dodge, 4 weapons, all prompts, 3 enemies, 4-phase boss, pickups, Data/Humanity shrines, key gate, HUD, full menus), held back only by zero automated tests. | Issues: No tests (tests/ empty; only data-testid attrs). OPEN prompt unseals boss gate with no proximity check to the gate (Logic.jsx:262). Backend CORS allow_credentials with wildcard origins (server.py:72), though backend is unused by the game.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8073,6 +9943,253 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="95" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Large deviations &amp; WHY — so no number looks like unexplained noise (root cause from trajectory + LLM-call data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Deviation</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Magnitude</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Why (root cause from data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>Cross-arm</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Normal ECU 23.7 vs eph3 12.5</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>1.9x</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
+          <t>Normal self-decides scope and builds broader before previewing (more steps); eph3/v2 MVP-split build a focused Phase-1 first. Quality stays ~equal (Normal 6.7 / eph3 7.0), so eph3 is cheaper for the same quality.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Cross-arm</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Normal ECU 45.3 vs v2 20.0</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>2.3x</t>
+        </is>
+      </c>
+      <c r="E5" s="20" t="inlineStr">
+        <is>
+          <t>Micro-loans is the heaviest prompt. Normal attempts the full module set (88-108 LLM calls, deep build) -&gt; 45 ECU; v2 credit-cap forces a leaner MVP -&gt; 20 ECU but lower quality (6.0 vs Normal 6.3 / eph3 8.0). eph3 mid-cost (31.6) with best quality (8.0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Cross-arm</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>eph3 ECU 39.3 vs v2 14.8</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>2.7x</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>eph3 3D-game builds (escape-cathedral 50.5, context-zero-6 58.2) ran 116-124 LLM calls + 17-30 screenshots = heavy Three.js visual-iteration/polish loops. v2 P5 builds were leaner (29-38 calls) and STARTED (stopped earlier). Also small-n: eph3 has 3 P5, v2 only 2. Cost here is iteration depth, not the prompt arm itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Within-arm</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>eph3: dialogist-fight-3 9.2 vs siblings ~50</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>0.2x median</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Stopped early (STARTED state, only 22 LLM calls / 19 steps) vs escape-cathedral 124 calls &amp; context-zero-6 116 calls. It built less iteration, so cheap but the least-polished of the three (code systems still present).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="58" customHeight="1">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Within-arm</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Normal: dialogist-fight-1 34.0 vs siblings ~19</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>1.7x median</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>More visual iteration: 10 screenshots / 94 LLM calls vs context-zero-3 (18.6 ECU) &amp; prompt-cathedral (20.1). The agent looped on rendering/combat polish.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Within-arm</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Normal: rendoc-loans-4 50.5 (highest single ECU)</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>top of P3</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>93 LLM calls + 22 calls &gt;30s + 1 hit the 600s timeout (hang+retry). Deepest build of the loan dashboards; the timeout-retry added latency and cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="58" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Consistency</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>eph3 ECU std-dev 21.5 (vs v2 3.4)</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>widest spread</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Driven entirely by the two heavy 3D builds (50-58 ECU) vs the early-stopped dialogist-fight-3 (9.2). 3D/game prompts have the least predictable cost across all arms.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8163,7 +10280,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="25" t="inlineStr">
         <is>
           <t>https://kanban-sync.stage-preview.emergentagent.com</t>
         </is>
@@ -8195,7 +10312,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="25" t="inlineStr">
         <is>
           <t>https://project-sync.stage-preview.emergentagent.com</t>
         </is>
@@ -8227,7 +10344,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E7" s="25" t="inlineStr">
         <is>
           <t>https://task-flow-57.stage-preview.emergentagent.com</t>
         </is>
@@ -8259,7 +10376,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="25" t="inlineStr">
         <is>
           <t>https://project-hub-25.stage-preview.emergentagent.com</t>
         </is>
@@ -8291,7 +10408,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="25" t="inlineStr">
         <is>
           <t>https://teamtask-1.stage-preview.emergentagent.com</t>
         </is>
@@ -8323,7 +10440,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="25" t="inlineStr">
         <is>
           <t>https://workflow-central-2.stage-preview.emergentagent.com</t>
         </is>
@@ -8355,7 +10472,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="25" t="inlineStr">
         <is>
           <t>https://kanban-pro-3.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -8387,7 +10504,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="25" t="inlineStr">
         <is>
           <t>https://project-flow-9.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -8419,7 +10536,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>https://workflow-pro-6.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -8500,7 +10617,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>https://booth-planner-1.stage-preview.emergentagent.com</t>
         </is>
@@ -8532,7 +10649,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>https://event-profit-hub.stage-preview.emergentagent.com</t>
         </is>
@@ -8564,7 +10681,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="25" t="inlineStr">
         <is>
           <t>https://know-before-show-1.stage-preview.emergentagent.com</t>
         </is>
@@ -8596,7 +10713,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t>https://know-before-show-2.stage-preview.emergentagent.com</t>
         </is>
@@ -8628,7 +10745,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E21" s="24" t="inlineStr">
+      <c r="E21" s="25" t="inlineStr">
         <is>
           <t>https://profit-prep.stage-preview.emergentagent.com</t>
         </is>
@@ -8660,7 +10777,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E22" s="25" t="inlineStr">
         <is>
           <t>https://vendor-calculator-4.stage-preview.emergentagent.com</t>
         </is>
@@ -8692,7 +10809,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t>https://know-before-show-5.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -8724,7 +10841,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="E24" s="25" t="inlineStr">
         <is>
           <t>https://profit-estimator-1.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -8756,7 +10873,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E25" s="24" t="inlineStr">
+      <c r="E25" s="25" t="inlineStr">
         <is>
           <t>https://profit-estimator-2.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -8837,7 +10954,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E29" s="24" t="inlineStr">
+      <c r="E29" s="25" t="inlineStr">
         <is>
           <t>https://credit-control.stage-preview.emergentagent.com</t>
         </is>
@@ -8869,7 +10986,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E30" s="24" t="inlineStr">
+      <c r="E30" s="25" t="inlineStr">
         <is>
           <t>https://micro-lending-hub.stage-preview.emergentagent.com</t>
         </is>
@@ -8901,7 +11018,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E31" s="24" t="inlineStr">
+      <c r="E31" s="25" t="inlineStr">
         <is>
           <t>https://rendoc-loans-4.stage-preview.emergentagent.com</t>
         </is>
@@ -8933,7 +11050,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E32" s="24" t="inlineStr">
+      <c r="E32" s="25" t="inlineStr">
         <is>
           <t>https://micro-loans-admin.stage-preview.emergentagent.com</t>
         </is>
@@ -8965,7 +11082,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E33" s="24" t="inlineStr">
+      <c r="E33" s="25" t="inlineStr">
         <is>
           <t>https://rendoc-credit-1.stage-preview.emergentagent.com</t>
         </is>
@@ -8997,7 +11114,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E34" s="24" t="inlineStr">
+      <c r="E34" s="25" t="inlineStr">
         <is>
           <t>https://rendoc-portfolio.stage-preview.emergentagent.com</t>
         </is>
@@ -9029,7 +11146,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E35" s="24" t="inlineStr">
+      <c r="E35" s="25" t="inlineStr">
         <is>
           <t>https://micro-lend-hub.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9061,7 +11178,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E36" s="24" t="inlineStr">
+      <c r="E36" s="25" t="inlineStr">
         <is>
           <t>https://portfolio-pilot.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9093,7 +11210,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E37" s="24" t="inlineStr">
+      <c r="E37" s="25" t="inlineStr">
         <is>
           <t>https://rendoc-loans-8.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9174,7 +11291,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E41" s="24" t="inlineStr">
+      <c r="E41" s="25" t="inlineStr">
         <is>
           <t>https://custom-proof.stage-preview.emergentagent.com</t>
         </is>
@@ -9206,7 +11323,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E42" s="24" t="inlineStr">
+      <c r="E42" s="25" t="inlineStr">
         <is>
           <t>https://engrave-studio-3.stage-preview.emergentagent.com</t>
         </is>
@@ -9238,7 +11355,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E43" s="24" t="inlineStr">
+      <c r="E43" s="25" t="inlineStr">
         <is>
           <t>https://vector-create.stage-preview.emergentagent.com</t>
         </is>
@@ -9270,7 +11387,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E44" s="24" t="inlineStr">
+      <c r="E44" s="25" t="inlineStr">
         <is>
           <t>https://create-ship-direct.stage-preview.emergentagent.com</t>
         </is>
@@ -9302,7 +11419,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E45" s="24" t="inlineStr">
+      <c r="E45" s="25" t="inlineStr">
         <is>
           <t>https://custom-maker.stage-preview.emergentagent.com</t>
         </is>
@@ -9334,7 +11451,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E46" s="24" t="inlineStr">
+      <c r="E46" s="25" t="inlineStr">
         <is>
           <t>https://design-to-print-1.stage-preview.emergentagent.com</t>
         </is>
@@ -9366,7 +11483,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E47" s="24" t="inlineStr">
+      <c r="E47" s="25" t="inlineStr">
         <is>
           <t>https://engrave-studio-4.stage-preview.emergentagent.com</t>
         </is>
@@ -9398,7 +11515,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E48" s="24" t="inlineStr">
+      <c r="E48" s="25" t="inlineStr">
         <is>
           <t>https://engrave-studio-5.stage-preview.emergentagent.com</t>
         </is>
@@ -9430,7 +11547,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E49" s="24" t="inlineStr">
+      <c r="E49" s="25" t="inlineStr">
         <is>
           <t>https://personalize-now.stage-preview.emergentagent.com</t>
         </is>
@@ -9462,7 +11579,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E50" s="24" t="inlineStr">
+      <c r="E50" s="25" t="inlineStr">
         <is>
           <t>https://design-engrave.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9494,7 +11611,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E51" s="24" t="inlineStr">
+      <c r="E51" s="25" t="inlineStr">
         <is>
           <t>https://personalize-pro-1.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9575,7 +11692,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E55" s="24" t="inlineStr">
+      <c r="E55" s="25" t="inlineStr">
         <is>
           <t>https://context-zero-3.stage-preview.emergentagent.com</t>
         </is>
@@ -9607,7 +11724,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E56" s="24" t="inlineStr">
+      <c r="E56" s="25" t="inlineStr">
         <is>
           <t>https://dialogist-fight-1.stage-preview.emergentagent.com</t>
         </is>
@@ -9639,7 +11756,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E57" s="24" t="inlineStr">
+      <c r="E57" s="25" t="inlineStr">
         <is>
           <t>https://prompt-cathedral.stage-preview.emergentagent.com</t>
         </is>
@@ -9671,7 +11788,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="E58" s="24" t="inlineStr">
+      <c r="E58" s="25" t="inlineStr">
         <is>
           <t>https://context-zero-5.stage-preview.emergentagent.com</t>
         </is>
@@ -9703,7 +11820,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="E59" s="24" t="inlineStr">
+      <c r="E59" s="25" t="inlineStr">
         <is>
           <t>https://escape-ai.stage-preview.emergentagent.com</t>
         </is>
@@ -9735,7 +11852,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E60" s="24" t="inlineStr">
+      <c r="E60" s="25" t="inlineStr">
         <is>
           <t>https://context-zero-6.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9767,7 +11884,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="E61" s="24" t="inlineStr">
+      <c r="E61" s="25" t="inlineStr">
         <is>
           <t>https://dialogist-fight-3.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9799,7 +11916,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="E62" s="24" t="inlineStr">
+      <c r="E62" s="25" t="inlineStr">
         <is>
           <t>https://escape-cathedral.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -9871,7 +11988,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9977,7 +12094,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="H4" s="25" t="inlineStr">
         <is>
           <t>https://kanban-sync.stage-preview.emergentagent.com</t>
         </is>
@@ -10016,7 +12133,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="25" t="inlineStr">
         <is>
           <t>https://teamtask-1.stage-preview.emergentagent.com</t>
         </is>
@@ -10055,7 +12172,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H6" s="24" t="inlineStr">
+      <c r="H6" s="25" t="inlineStr">
         <is>
           <t>https://workflow-pro-6.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -10094,7 +12211,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H8" s="24" t="inlineStr">
+      <c r="H8" s="25" t="inlineStr">
         <is>
           <t>https://booth-planner-1.stage-preview.emergentagent.com</t>
         </is>
@@ -10133,7 +12250,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H9" s="24" t="inlineStr">
+      <c r="H9" s="25" t="inlineStr">
         <is>
           <t>https://profit-prep.stage-preview.emergentagent.com</t>
         </is>
@@ -10172,7 +12289,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H10" s="24" t="inlineStr">
+      <c r="H10" s="25" t="inlineStr">
         <is>
           <t>https://profit-estimator-2.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -10211,7 +12328,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H12" s="24" t="inlineStr">
+      <c r="H12" s="25" t="inlineStr">
         <is>
           <t>https://rendoc-loans-4.stage-preview.emergentagent.com</t>
         </is>
@@ -10250,7 +12367,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H13" s="24" t="inlineStr">
+      <c r="H13" s="25" t="inlineStr">
         <is>
           <t>https://rendoc-credit-1.stage-preview.emergentagent.com</t>
         </is>
@@ -10289,7 +12406,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H14" s="24" t="inlineStr">
+      <c r="H14" s="25" t="inlineStr">
         <is>
           <t>https://micro-lend-hub.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -10328,7 +12445,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="H16" s="25" t="inlineStr">
         <is>
           <t>https://custom-proof.stage-preview.emergentagent.com</t>
         </is>
@@ -10367,7 +12484,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H17" s="24" t="inlineStr">
+      <c r="H17" s="25" t="inlineStr">
         <is>
           <t>https://design-to-print-1.stage-preview.emergentagent.com</t>
         </is>
@@ -10406,7 +12523,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H18" s="24" t="inlineStr">
+      <c r="H18" s="25" t="inlineStr">
         <is>
           <t>https://design-engrave.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -10445,7 +12562,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H20" s="24" t="inlineStr">
+      <c r="H20" s="25" t="inlineStr">
         <is>
           <t>https://dialogist-fight-1.stage-preview.emergentagent.com</t>
         </is>
@@ -10484,7 +12601,7 @@
           <t>STARTED</t>
         </is>
       </c>
-      <c r="H21" s="24" t="inlineStr">
+      <c r="H21" s="25" t="inlineStr">
         <is>
           <t>https://context-zero-5.stage-preview.emergentagent.com</t>
         </is>
@@ -10523,7 +12640,7 @@
           <t>RESUMED</t>
         </is>
       </c>
-      <c r="H22" s="24" t="inlineStr">
+      <c r="H22" s="25" t="inlineStr">
         <is>
           <t>https://escape-cathedral.internal.stage-preview.emergentagent.com</t>
         </is>
@@ -10555,7 +12672,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13375,1870 +15492,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L47"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="6" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="6" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="90" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>Arm</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>Prompt</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>Slug</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>Spec</t>
-        </is>
-      </c>
-      <c r="E1" s="4" t="inlineStr">
-        <is>
-          <t>Arch</t>
-        </is>
-      </c>
-      <c r="F1" s="4" t="inlineStr">
-        <is>
-          <t>Err</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Sec</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Qual</t>
-        </is>
-      </c>
-      <c r="I1" s="4" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-      <c r="J1" s="4" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="K1" s="4" t="inlineStr">
-        <is>
-          <t>Tier</t>
-        </is>
-      </c>
-      <c r="L1" s="4" t="inlineStr">
-        <is>
-          <t>Verdict / Top issues</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>kanban-sync</t>
-        </is>
-      </c>
-      <c r="D2" s="14" t="inlineStr"/>
-      <c r="E2" s="14" t="inlineStr"/>
-      <c r="F2" s="14" t="inlineStr"/>
-      <c r="G2" s="14" t="inlineStr"/>
-      <c r="H2" s="14" t="inlineStr"/>
-      <c r="I2" s="14" t="inlineStr"/>
-      <c r="J2" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K2" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L2" s="20" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
-        <is>
-          <t>project-sync</t>
-        </is>
-      </c>
-      <c r="D3" s="14" t="inlineStr"/>
-      <c r="E3" s="14" t="inlineStr"/>
-      <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="14" t="inlineStr"/>
-      <c r="H3" s="14" t="inlineStr"/>
-      <c r="I3" s="14" t="inlineStr"/>
-      <c r="J3" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K3" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L3" s="20" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C4" s="17" t="inlineStr">
-        <is>
-          <t>task-flow-57</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr"/>
-      <c r="E4" s="14" t="inlineStr"/>
-      <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="14" t="inlineStr"/>
-      <c r="H4" s="14" t="inlineStr"/>
-      <c r="I4" s="14" t="inlineStr"/>
-      <c r="J4" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L4" s="20" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>booth-planner-1</t>
-        </is>
-      </c>
-      <c r="D5" s="14" t="inlineStr"/>
-      <c r="E5" s="14" t="inlineStr"/>
-      <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="14" t="inlineStr"/>
-      <c r="H5" s="14" t="inlineStr"/>
-      <c r="I5" s="14" t="inlineStr"/>
-      <c r="J5" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K5" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L5" s="20" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>event-profit-hub</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr"/>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="14" t="inlineStr"/>
-      <c r="H6" s="14" t="inlineStr"/>
-      <c r="I6" s="14" t="inlineStr"/>
-      <c r="J6" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L6" s="20" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>know-before-show-1</t>
-        </is>
-      </c>
-      <c r="D7" s="14" t="inlineStr"/>
-      <c r="E7" s="14" t="inlineStr"/>
-      <c r="F7" s="14" t="inlineStr"/>
-      <c r="G7" s="14" t="inlineStr"/>
-      <c r="H7" s="14" t="inlineStr"/>
-      <c r="I7" s="14" t="inlineStr"/>
-      <c r="J7" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K7" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L7" s="20" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>credit-control</t>
-        </is>
-      </c>
-      <c r="D8" s="14" t="inlineStr"/>
-      <c r="E8" s="14" t="inlineStr"/>
-      <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr"/>
-      <c r="H8" s="14" t="inlineStr"/>
-      <c r="I8" s="14" t="inlineStr"/>
-      <c r="J8" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K8" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L8" s="20" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>micro-lending-hub</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr"/>
-      <c r="E9" s="14" t="inlineStr"/>
-      <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="14" t="inlineStr"/>
-      <c r="H9" s="14" t="inlineStr"/>
-      <c r="I9" s="14" t="inlineStr"/>
-      <c r="J9" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K9" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L9" s="20" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>rendoc-loans-4</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr"/>
-      <c r="H10" s="14" t="inlineStr"/>
-      <c r="I10" s="14" t="inlineStr"/>
-      <c r="J10" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L10" s="20" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C11" s="17" t="inlineStr">
-        <is>
-          <t>custom-proof</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr"/>
-      <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="14" t="inlineStr"/>
-      <c r="H11" s="14" t="inlineStr"/>
-      <c r="I11" s="14" t="inlineStr"/>
-      <c r="J11" s="14" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="K11" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L11" s="20" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>engrave-studio-3</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr"/>
-      <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr"/>
-      <c r="H12" s="14" t="inlineStr"/>
-      <c r="I12" s="14" t="inlineStr"/>
-      <c r="J12" s="14" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L12" s="20" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>vector-create</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr"/>
-      <c r="E13" s="14" t="inlineStr"/>
-      <c r="F13" s="14" t="inlineStr"/>
-      <c r="G13" s="14" t="inlineStr"/>
-      <c r="H13" s="14" t="inlineStr"/>
-      <c r="I13" s="14" t="inlineStr"/>
-      <c r="J13" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K13" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L13" s="20" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>context-zero-3</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F14" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G14" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H14" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I14" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K14" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L14" s="20" t="inlineStr">
-        <is>
-          <t>A polished, feature-complete 3D roguelike vertical slice that covers nearly every spec system with clean engine/UI separation, let down only by a total absence of tests and a vanilla-Three.js (not R3F) implementation. | Issues: Zero tests (empty __init__.py only). Uses globals window.__msgTimer/__dlgTimer (engine.js bridged in Game.jsx:26-32). 1831-line monolith engine. No React error boundary; SSR-off via dynamic import only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="inlineStr">
-        <is>
-          <t>dialogist-fight-1</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F15" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K15" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L15" s="20" t="inlineStr">
-        <is>
-          <t>A near-complete, well-structured 3D roguelike that covers nearly every spec system with clean code, held back only by zero automated tests and a few minor dead-code/misleading-UI bugs. | Issues: No tests at all (empty tests dir, template test_result.md). Backend CORS '*' + allow_credentials (unused boilerplate). Dead code: unused dist2, empty gate-poll interval, magic-string 'gate' in castPrompt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Normal (eph1/gflash)</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>prompt-cathedral</t>
-        </is>
-      </c>
-      <c r="D16" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F16" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G16" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="H16" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I16" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K16" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L16" s="20" t="inlineStr">
-        <is>
-          <t>A feature-complete, well-architected R3F roguelike covering nearly every spec system (movement, dodge, 4 weapons, all prompts, 3 enemies, 4-phase boss, shrines, Model Key gate, full menus), held back only by zero tests and a Next.js-vs-CRA stack deviation. | Issues: No tests at all (empty tests/). Backend CORS allow_credentials=True with '*' origin and os.environ['MONGO_URL'] KeyError risk (dead code). HUD subscribes to full store + per-frame rAF force re-render; updatePickups no-op.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>project-hub-25</t>
-        </is>
-      </c>
-      <c r="D17" s="14" t="inlineStr"/>
-      <c r="E17" s="14" t="inlineStr"/>
-      <c r="F17" s="14" t="inlineStr"/>
-      <c r="G17" s="14" t="inlineStr"/>
-      <c r="H17" s="14" t="inlineStr"/>
-      <c r="I17" s="14" t="inlineStr"/>
-      <c r="J17" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="K17" s="14" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="L17" s="20" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>teamtask-1</t>
-        </is>
-      </c>
-      <c r="D18" s="14" t="inlineStr"/>
-      <c r="E18" s="14" t="inlineStr"/>
-      <c r="F18" s="14" t="inlineStr"/>
-      <c r="G18" s="14" t="inlineStr"/>
-      <c r="H18" s="14" t="inlineStr"/>
-      <c r="I18" s="14" t="inlineStr"/>
-      <c r="J18" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="K18" s="14" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="L18" s="20" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>workflow-central-2</t>
-        </is>
-      </c>
-      <c r="D19" s="14" t="inlineStr"/>
-      <c r="E19" s="14" t="inlineStr"/>
-      <c r="F19" s="14" t="inlineStr"/>
-      <c r="G19" s="14" t="inlineStr"/>
-      <c r="H19" s="14" t="inlineStr"/>
-      <c r="I19" s="14" t="inlineStr"/>
-      <c r="J19" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="K19" s="14" t="inlineStr">
-        <is>
-          <t>Weak</t>
-        </is>
-      </c>
-      <c r="L19" s="20" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>know-before-show-2</t>
-        </is>
-      </c>
-      <c r="D20" s="14" t="inlineStr"/>
-      <c r="E20" s="14" t="inlineStr"/>
-      <c r="F20" s="14" t="inlineStr"/>
-      <c r="G20" s="14" t="inlineStr"/>
-      <c r="H20" s="14" t="inlineStr"/>
-      <c r="I20" s="14" t="inlineStr"/>
-      <c r="J20" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K20" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L20" s="20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>profit-prep</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr"/>
-      <c r="E21" s="14" t="inlineStr"/>
-      <c r="F21" s="14" t="inlineStr"/>
-      <c r="G21" s="14" t="inlineStr"/>
-      <c r="H21" s="14" t="inlineStr"/>
-      <c r="I21" s="14" t="inlineStr"/>
-      <c r="J21" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K21" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L21" s="20" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>vendor-calculator-4</t>
-        </is>
-      </c>
-      <c r="D22" s="14" t="inlineStr"/>
-      <c r="E22" s="14" t="inlineStr"/>
-      <c r="F22" s="14" t="inlineStr"/>
-      <c r="G22" s="14" t="inlineStr"/>
-      <c r="H22" s="14" t="inlineStr"/>
-      <c r="I22" s="14" t="inlineStr"/>
-      <c r="J22" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K22" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L22" s="20" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>micro-loans-admin</t>
-        </is>
-      </c>
-      <c r="D23" s="14" t="inlineStr"/>
-      <c r="E23" s="14" t="inlineStr"/>
-      <c r="F23" s="14" t="inlineStr"/>
-      <c r="G23" s="14" t="inlineStr"/>
-      <c r="H23" s="14" t="inlineStr"/>
-      <c r="I23" s="14" t="inlineStr"/>
-      <c r="J23" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K23" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L23" s="20" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>rendoc-credit-1</t>
-        </is>
-      </c>
-      <c r="D24" s="14" t="inlineStr"/>
-      <c r="E24" s="14" t="inlineStr"/>
-      <c r="F24" s="14" t="inlineStr"/>
-      <c r="G24" s="14" t="inlineStr"/>
-      <c r="H24" s="14" t="inlineStr"/>
-      <c r="I24" s="14" t="inlineStr"/>
-      <c r="J24" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K24" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L24" s="20" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>rendoc-portfolio</t>
-        </is>
-      </c>
-      <c r="D25" s="14" t="inlineStr"/>
-      <c r="E25" s="14" t="inlineStr"/>
-      <c r="F25" s="14" t="inlineStr"/>
-      <c r="G25" s="14" t="inlineStr"/>
-      <c r="H25" s="14" t="inlineStr"/>
-      <c r="I25" s="14" t="inlineStr"/>
-      <c r="J25" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K25" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L25" s="20" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>create-ship-direct</t>
-        </is>
-      </c>
-      <c r="D26" s="14" t="inlineStr"/>
-      <c r="E26" s="14" t="inlineStr"/>
-      <c r="F26" s="14" t="inlineStr"/>
-      <c r="G26" s="14" t="inlineStr"/>
-      <c r="H26" s="14" t="inlineStr"/>
-      <c r="I26" s="14" t="inlineStr"/>
-      <c r="J26" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K26" s="14" t="inlineStr">
-        <is>
-          <t>Solid</t>
-        </is>
-      </c>
-      <c r="L26" s="20" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>custom-maker</t>
-        </is>
-      </c>
-      <c r="D27" s="14" t="inlineStr"/>
-      <c r="E27" s="14" t="inlineStr"/>
-      <c r="F27" s="14" t="inlineStr"/>
-      <c r="G27" s="14" t="inlineStr"/>
-      <c r="H27" s="14" t="inlineStr"/>
-      <c r="I27" s="14" t="inlineStr"/>
-      <c r="J27" s="14" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="K27" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L27" s="20" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B28" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>design-to-print-1</t>
-        </is>
-      </c>
-      <c r="D28" s="14" t="inlineStr"/>
-      <c r="E28" s="14" t="inlineStr"/>
-      <c r="F28" s="14" t="inlineStr"/>
-      <c r="G28" s="14" t="inlineStr"/>
-      <c r="H28" s="14" t="inlineStr"/>
-      <c r="I28" s="14" t="inlineStr"/>
-      <c r="J28" s="14" t="n">
-        <v>7.7</v>
-      </c>
-      <c r="K28" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L28" s="20" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>engrave-studio-4</t>
-        </is>
-      </c>
-      <c r="D29" s="14" t="inlineStr"/>
-      <c r="E29" s="14" t="inlineStr"/>
-      <c r="F29" s="14" t="inlineStr"/>
-      <c r="G29" s="14" t="inlineStr"/>
-      <c r="H29" s="14" t="inlineStr"/>
-      <c r="I29" s="14" t="inlineStr"/>
-      <c r="J29" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="K29" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L29" s="20" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>engrave-studio-5</t>
-        </is>
-      </c>
-      <c r="D30" s="14" t="inlineStr"/>
-      <c r="E30" s="14" t="inlineStr"/>
-      <c r="F30" s="14" t="inlineStr"/>
-      <c r="G30" s="14" t="inlineStr"/>
-      <c r="H30" s="14" t="inlineStr"/>
-      <c r="I30" s="14" t="inlineStr"/>
-      <c r="J30" s="14" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K30" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L30" s="20" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="inlineStr">
-        <is>
-          <t>personalize-now</t>
-        </is>
-      </c>
-      <c r="D31" s="14" t="inlineStr"/>
-      <c r="E31" s="14" t="inlineStr"/>
-      <c r="F31" s="14" t="inlineStr"/>
-      <c r="G31" s="14" t="inlineStr"/>
-      <c r="H31" s="14" t="inlineStr"/>
-      <c r="I31" s="14" t="inlineStr"/>
-      <c r="J31" s="14" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="K31" s="14" t="inlineStr">
-        <is>
-          <t>Mid</t>
-        </is>
-      </c>
-      <c r="L31" s="20" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>context-zero-5</t>
-        </is>
-      </c>
-      <c r="D32" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E32" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F32" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G32" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H32" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I32" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K32" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L32" s="20" t="inlineStr">
-        <is>
-          <t>A near-complete, well-structured vertical slice that implements virtually the entire spec (movement, dodge, 4 weapons, 4 prompts, 3 enemy types, multi-phase Dialogist boss, pickups, dual upgrade shrine, Model Key gate, connected chambers, full HUD and menus) in clean R3F code, held back mainly by zero automated tests. | Issues: .env committed and not gitignored (localhost Mongo only). CORS defaults to '*' with Allow-Credentials true. State bridged via window.__contextZero global. Dead pickup branches (memory/data never spawned).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>v2_credit_cap (eph2)</t>
-        </is>
-      </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C33" s="17" t="inlineStr">
-        <is>
-          <t>escape-ai</t>
-        </is>
-      </c>
-      <c r="D33" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E33" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F33" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="H33" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="I33" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K33" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L33" s="20" t="inlineStr">
-        <is>
-          <t>A feature-complete, well-structured R3F roguelike covering every spec system (movement, dodge, 4 weapons, 4 prompts, 3 enemies, 4-phase Dialogist, pickups, Data/Humanity shrines, chambers, Model Key gate, full menus) but ships with zero automated tests. | Issues: No tests at all (empty tests/, template test_result.md). Dead code: store.js:319-322 STUN loop does nothing, empty mouse branch. window.__cz_castStun global coupling; boss hardcoded at origin; ~50 unused shadcn components.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C34" s="17" t="inlineStr">
-        <is>
-          <t>kanban-pro-3</t>
-        </is>
-      </c>
-      <c r="D34" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="E34" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F34" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G34" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="H34" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I34" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="J34" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K34" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L34" s="20" t="inlineStr">
-        <is>
-          <t>A polished, clean implementation of the core CRUD/kanban/dashboard slice with excellent drag-drop and tested isolation, but roughly half the spec breadth (subtasks, comments, search, calendar, dark mode, notifications) is missing. | Issues: CORS allow_origins='*' with allow_credentials=True (insecure/invalid combo); no frontend tests; ~6 spec features absent in both API and UI.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C35" s="17" t="inlineStr">
-        <is>
-          <t>project-flow-9</t>
-        </is>
-      </c>
-      <c r="D35" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="E35" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F35" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="H35" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I35" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="J35" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K35" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L35" s="20" t="inlineStr">
-        <is>
-          <t>A clean, well-architected MVP covering auth, projects, task CRUD with properties, kanban drag-drop and dashboard, but it omits roughly half the spec (subtasks, comments, search/filter, calendar, dark mode, notifications). | Issues: CORS allow_origins='*' with allow_credentials=True (env default). Reorder endpoint loops per-item awaits (N writes) without bulk_write. No rate limiting on auth. middleware added after include_router.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="C36" s="17" t="inlineStr">
-        <is>
-          <t>workflow-pro-6</t>
-        </is>
-      </c>
-      <c r="D36" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F36" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H36" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I36" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="J36" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K36" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L36" s="20" t="inlineStr">
-        <is>
-          <t>A clean, well-architected core (auth, task CRUD with properties, owner-scoped queries, polished dnd-kit kanban, dashboard, real backend tests) that omits roughly half the spec's distinctive features—subtasks, comments, calendar, notifications, dark-mode toggle. | Issues: CORS allow_origins='*' with allow_credentials=True (browsers reject; insecure). No login rate limiting. update_task (server.py:316-322) has duplicated/confusing merge logic. due_date stored as string, compared lexicographically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C37" s="17" t="inlineStr">
-        <is>
-          <t>know-before-show-5</t>
-        </is>
-      </c>
-      <c r="D37" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E37" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="F37" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G37" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="H37" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I37" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="J37" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K37" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L37" s="20" t="inlineStr">
-        <is>
-          <t>A polished, feature-complete localStorage-only vendor profit app with sound calculator math, full planner/checklist/dashboard, and clean architecture, held back only by a total absence of frontend tests. | Issues: No frontend tests despite easily testable pure fns (calculator.js, storage.js). Minor: unused imports in Planner; shadowed `num` in formatCurrency; no try/catch on localStorage write (quota).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C38" s="17" t="inlineStr">
-        <is>
-          <t>profit-estimator-1</t>
-        </is>
-      </c>
-      <c r="D38" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E38" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F38" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G38" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="H38" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I38" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="J38" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K38" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L38" s="20" t="inlineStr">
-        <is>
-          <t>A clean, fully spec-compliant mobile-first vendor profit app with correct calculator math, full planner, exact 21-item checklist, aggregating dashboard, robust localStorage, and Verbum footer—held back only by zero tests and minor dead code. | Issues: Dashboard.jsx:213-214 dead hidden input sums ev.profitEstimate, a field Planner never writes. tests/ empty—no unit tests for calc math. Dashboard state only read on mount, may show stale data.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C39" s="17" t="inlineStr">
-        <is>
-          <t>profit-estimator-2</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E39" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F39" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G39" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="H39" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I39" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K39" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L39" s="20" t="inlineStr">
-        <is>
-          <t>A clean, complete, well-structured mobile-first localStorage vendor profit app that covers every spec feature with readable code, though it ships no automated tests. | Issues: No real tests (tests/__init__.py empty). num() silently coerces bad input to 0 with no negative-value guard beyond HTML min. Dashboard upcoming-event date filter is timezone-sensitive (new Date('YYYY-MM-DD')).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C40" s="17" t="inlineStr">
-        <is>
-          <t>micro-lend-hub</t>
-        </is>
-      </c>
-      <c r="D40" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E40" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="F40" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G40" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H40" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I40" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="J40" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K40" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L40" s="20" t="inlineStr">
-        <is>
-          <t>A comprehensive, well-architected micro-loans dashboard covering the full spec with clean modular routes, RBAC, risk scoring, and audit logging, held back mainly by CORS/secret hardening gaps. | Issues: CORS allow_origins=* with allow_credentials=True (server.py:80-86); hardcoded JWT_SECRET fallback (auth.py:13); public /applications/intake unbounded; tests are live-URL integration only, no risk-engine unit tests.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C41" s="17" t="inlineStr">
-        <is>
-          <t>portfolio-pilot</t>
-        </is>
-      </c>
-      <c r="D41" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="E41" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F41" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="G41" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H41" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I41" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="J41" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K41" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L41" s="20" t="inlineStr">
-        <is>
-          <t>A cohesive, well-structured RENDOC micro-loans dashboard covering nearly the entire spec with real RBAC, risk scoring, amortization, collections, audit log and strong integration tests, marred mainly by a stubbed document upload and thin frontend fetch error handling. | Issues: Document upload is a placeholder despite being in spec; frontend load() fetchers lack try/catch (perpetual "Loading"); unauthenticated /seed?force=true wipes all data; CORS=* with allow_credentials.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="C42" s="17" t="inlineStr">
-        <is>
-          <t>rendoc-loans-8</t>
-        </is>
-      </c>
-      <c r="D42" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E42" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F42" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G42" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H42" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I42" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="J42" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K42" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L42" s="20" t="inlineStr">
-        <is>
-          <t>A thorough, well-structured full-stack loans platform covering nearly the entire spec (RBAC, pipeline, risk scoring, lifecycle, collections, audit) with broad passing integration tests, held back only by a few security defaults. | Issues: JWT_SECRET hardcoded dev fallback (auth.py:10); CORS allow_origins=* with allow_credentials=True (server.py:1435); upload stores raw file.filename - path traversal risk (server.py:724); reads not scoped to owning officer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C43" s="17" t="inlineStr">
-        <is>
-          <t>design-engrave</t>
-        </is>
-      </c>
-      <c r="D43" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E43" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="F43" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G43" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H43" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I43" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="J43" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K43" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L43" s="20" t="inlineStr">
-        <is>
-          <t>A cohesive, well-architected laser-engraving customizer that covers nearly the full spec with a strong live 2D proof flow, production queue, and passing integration tests; main gap is server-side trust of client-supplied prices. | Issues: Server trusts client unit_price/subtotal/total (models.py:93-101); CORS allow_origins=* with allow_credentials=True (server.py:240); default JWT secret in committed .env; GET /orders/{id} unauthenticated (server.py:169).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B44" s="14" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="C44" s="17" t="inlineStr">
-        <is>
-          <t>personalize-pro-1</t>
-        </is>
-      </c>
-      <c r="D44" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="E44" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="F44" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="G44" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H44" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I44" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="J44" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K44" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L44" s="20" t="inlineStr">
-        <is>
-          <t>A clean, cohesive laser-engraving MVP covering catalog, configurator, live 2D proof, volume pricing, checkout, kanban production queue and owner alerts, marred mainly by client-trusted pricing and wildcard CORS. | Issues: server.py:289 trusts client unit_price (price tampering, tiers not re-validated); CORS '*' + allow_credentials True (L594); JWT_SECRET hardcoded fallback (L35).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C45" s="17" t="inlineStr">
-        <is>
-          <t>context-zero-6</t>
-        </is>
-      </c>
-      <c r="D45" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F45" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G45" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H45" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="I45" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="K45" s="14" t="inlineStr">
-        <is>
-          <t>Acceptable</t>
-        </is>
-      </c>
-      <c r="L45" s="20" t="inlineStr">
-        <is>
-          <t>A complete, well-architected R3F roguelike covering nearly all spec systems (movement, dodge, 4 weapons, 4 enemy types, 4-phase boss, upgrades, key gate, HUD, menus), let down by a non-functional OPEN prompt and a total absence of tests. | Issues: No tests (empty tests/__init__.py, no frontend specs). Dead/abandoned code in levelGen.js:84-96. Boss collider sway math duplicated (Tick.jsx 701-715 vs 752-758). Backend CORS allow_origins='*' + allow_credentials=True (unused boilerplate).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>dialogist-fight-3</t>
-        </is>
-      </c>
-      <c r="D46" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E46" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="F46" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G46" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H46" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="I46" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K46" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L46" s="20" t="inlineStr">
-        <is>
-          <t>A feature-complete, well-structured 3D roguelike that delivers nearly every spec system (4-phase boss, prompts, 3 enemy types, key gate, dual-path upgrades, full menus) but ships with zero automated tests. | Issues: Empty tests/ dir, no test framework. Minor dead code: unused lineHitsWall, no-op SWARM?1:1 (gameplay.js:672), unused onPause prop, duplicate root route. CORS defaults to '*'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>eph3 (long-prompt-1)</t>
-        </is>
-      </c>
-      <c r="B47" s="14" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="C47" s="17" t="inlineStr">
-        <is>
-          <t>escape-cathedral</t>
-        </is>
-      </c>
-      <c r="D47" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="E47" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="F47" s="14" t="n">
-        <v>7</v>
-      </c>
-      <c r="G47" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="H47" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="I47" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="J47" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="K47" s="14" t="inlineStr">
-        <is>
-          <t>Strong</t>
-        </is>
-      </c>
-      <c r="L47" s="20" t="inlineStr">
-        <is>
-          <t>A near-complete, cleanly architected R3F roguelike covering essentially every spec system (movement, dodge, 4 weapons, all prompts, 3 enemies, 4-phase boss, pickups, Data/Humanity shrines, key gate, HUD, full menus), held back only by zero automated tests. | Issues: No tests (tests/ empty; only data-testid attrs). OPEN prompt unseals boss gate with no proximity check to the gate (Logic.jsx:262). Backend CORS allow_credentials with wildcard origins (server.py:72), though backend is unused by the game.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>